<commit_message>
progress: 41 village workbooks (randomwalk-TRX50-WS 2026-10-09T18:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chutalakuppam_13.406573_80.100795.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chutalakuppam_13.406573_80.100795.xlsx
@@ -650,11 +650,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -662,11 +657,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -674,11 +664,6 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>10A1, 10A2, 10A3, 10B, 11A, 11B, 1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -686,11 +671,6 @@
           <t>28</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>1A1A1, 1A2, 1B, 1C, 2, 3A, 3B, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -698,11 +678,6 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A, 1A1B, 1A2A1, 1A2B1, 1A3A, 1B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30A1, 30A2, 30B, 30C, 31, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -710,11 +685,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -722,11 +692,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1C1A1, 1C1A2, 1C2, 2A1A1A, 2A2, 2B, 3, 4, 5A, 5B, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -734,11 +699,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1A1, 1B, 2A1A, 2A2, 2B, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -746,11 +706,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>10, 16, 17, 18, 19, 1A1, 1A1B1, 1A2, 1B, 2, 20, 21A, 21B, 22, 23, 24, 25, 3, 4, 5A, 5B, 6, 7, 9</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -758,11 +713,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -770,11 +720,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -782,11 +727,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -794,11 +734,6 @@
           <t>36</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -806,11 +741,6 @@
           <t>37</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -818,11 +748,6 @@
           <t>38</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -830,11 +755,6 @@
           <t>39</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -842,11 +762,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -854,11 +769,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -866,11 +776,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -878,11 +783,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -890,11 +790,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1, 2, 3A1, 3A2, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -902,11 +797,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1, 2, 3A1A, 3A2, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -914,11 +804,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -926,11 +811,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -938,11 +818,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1TO3B</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -950,11 +825,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1ATO2</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -962,11 +832,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 20, 21, 22A, 22B, 22C, 23, 24A, 24B, 25, 26, 2A1A1A2A, 2A1A1B, 2A1A2, 2A1A3, 2A1A4, 2A1A5, 2A1B, 2A2, 2A3, 2A4, 2A5, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 2L, 3, 4, 5A1A1, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -974,11 +839,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -986,11 +846,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>1A1A1A, 1A1B, 1A2, 1A3, 1B, 1C1, 1C2, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1P, 1Q, 1R</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -998,11 +853,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 2A1A1A1A, 2A1B, 2A2, 2B, 2C, 2D, 2E, 2F, 2G, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1010,11 +860,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A1A1A, 1A1B, 1A1C, 1A2, 1B, 1C, 1D, 2, 20, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1022,11 +867,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 1A1A1A1A1, 1A1A1A2, 1A1A1B, 1A1A2, 1A1A3A, 1A1A4, 1A1B, 1A2A, 1A2B, 1A3, 1B, 1C, 1D, 2, 20, 21, 22, 23A, 23B, 24, 25, 3, 9</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1034,11 +874,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1046,11 +881,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1058,11 +888,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A10, 1A11, 1A12, 1A13, 1A1A1A1, 1A1A1B, 1A1A2, 1A1B, 1A1C, 1A1D, 1A1E, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9A, 1A9B, 2, 20, 21A, 21B, 22, 23, 24, 25, 3, 4, 5A, 5B, 5C</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1070,11 +895,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>1A1TO3B</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1082,11 +902,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>1ATO3</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1094,11 +909,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1TO9</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1106,11 +916,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1118,11 +923,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>1TO3</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1130,11 +930,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>1ATO4B</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1142,11 +937,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1TO10BTO15</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1154,11 +944,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>1TO3</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1166,11 +951,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 6</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1178,11 +958,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1TO4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1190,11 +965,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1202,11 +972,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1214,11 +979,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1226,11 +986,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1A, 2, 3, 4, 5, 6A, 9</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1238,11 +993,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1TO2F, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1250,11 +1000,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1TO3</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1262,11 +1007,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1274,21 +1014,11 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
           <t>74</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 43 village workbooks (randomwalk-TRX50-WS 2026-10-09T18:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chutalakuppam_13.406573_80.100795.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chutalakuppam_13.406573_80.100795.xlsx
@@ -650,6 +650,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -657,6 +662,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -664,6 +674,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10A3, 10B, 11A, 11B, 1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -671,6 +686,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A2, 1B, 1C, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -678,6 +698,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A, 1A1B, 1A2A1, 1A2B1, 1A3A, 1B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30A1, 30A2, 30B, 30C, 31, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -685,6 +710,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -692,6 +722,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1A1, 1C1A2, 1C2, 2A1A1A, 2A2, 2B, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -699,6 +734,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1A1, 1B, 2A1A, 2A2, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -706,6 +746,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10, 16, 17, 18, 19, 1A1, 1A1B1, 1A2, 1B, 2, 20, 21A, 21B, 22, 23, 24, 25, 3, 4, 5A, 5B, 6, 7, 9</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -713,6 +758,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -720,6 +770,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -727,6 +782,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -734,6 +794,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -741,6 +806,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -748,6 +818,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -755,6 +830,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -762,6 +842,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -769,6 +854,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -776,6 +866,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -783,6 +878,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -790,6 +890,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -797,6 +902,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1A, 3A2, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -804,6 +914,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -811,6 +926,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -818,6 +938,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1TO3B</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -825,6 +950,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1ATO2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -832,6 +962,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 20, 21, 22A, 22B, 22C, 23, 24A, 24B, 25, 26, 2A1A1A2A, 2A1A1B, 2A1A2, 2A1A3, 2A1A4, 2A1A5, 2A1B, 2A2, 2A3, 2A4, 2A5, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 2L, 3, 4, 5A1A1, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -839,6 +974,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -846,6 +986,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1B, 1A2, 1A3, 1B, 1C1, 1C2, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1P, 1Q, 1R</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -853,6 +998,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 2A1A1A1A, 2A1B, 2A2, 2B, 2C, 2D, 2E, 2F, 2G, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -860,6 +1010,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A1A1A, 1A1B, 1A1C, 1A2, 1B, 1C, 1D, 2, 20, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -867,6 +1022,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 1A1A1A1A1, 1A1A1A2, 1A1A1B, 1A1A2, 1A1A3A, 1A1A4, 1A1B, 1A2A, 1A2B, 1A3, 1B, 1C, 1D, 2, 20, 21, 22, 23A, 23B, 24, 25, 3, 9</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -874,6 +1034,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -881,6 +1046,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -888,6 +1058,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A10, 1A11, 1A12, 1A13, 1A1A1A1, 1A1A1B, 1A1A2, 1A1B, 1A1C, 1A1D, 1A1E, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9A, 1A9B, 2, 20, 21A, 21B, 22, 23, 24, 25, 3, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -895,6 +1070,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1A1TO3B</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -902,6 +1082,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1ATO3</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -909,6 +1094,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1TO9</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -916,6 +1106,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -923,6 +1118,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1TO3</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -930,6 +1130,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1ATO4B</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -937,6 +1142,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1TO10BTO15</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -944,6 +1154,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1TO3</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -951,6 +1166,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 6</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -958,6 +1178,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1TO4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -965,6 +1190,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -972,6 +1202,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -979,6 +1214,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -986,6 +1226,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1A, 2, 3, 4, 5, 6A, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -993,6 +1238,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1TO2F, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1000,6 +1250,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1TO3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1007,6 +1262,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1014,6 +1274,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1021,6 +1286,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1028,6 +1298,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1035,6 +1310,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1042,6 +1322,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1049,6 +1334,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1056,6 +1346,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1063,6 +1358,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1070,6 +1370,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1077,6 +1382,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1ATO2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1084,6 +1394,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1091,6 +1406,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1098,6 +1418,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1105,6 +1430,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1112,6 +1442,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1119,6 +1454,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1A, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1126,6 +1466,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1133,6 +1478,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1140,6 +1490,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I1A1A, 1I2, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1147,6 +1502,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1154,6 +1514,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1161,6 +1526,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1168,6 +1538,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1175,6 +1550,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1182,6 +1562,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1ATO5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1189,6 +1574,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1196,6 +1586,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1203,11 +1598,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1TO2C</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1ATO3</t>
         </is>
       </c>
     </row>

</xml_diff>